<commit_message>
Finalize MVA cloud reports and release artifacts
</commit_message>
<xml_diff>
--- a/output/excel/mva_crowdstrike_final_team_sample.xlsx
+++ b/output/excel/mva_crowdstrike_final_team_sample.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive Dashboard" sheetId="1" r:id="Racf03b5a09da4987"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monthly Dashboard" sheetId="2" r:id="R5239d2cdeec04484"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Adhoc Dashboard" sheetId="3" r:id="R04e6a03276284a69"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive Dashboard" sheetId="1" r:id="R674dcd0a08cc4d7d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monthly Dashboard" sheetId="2" r:id="Rb7e7139243e44fcf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Adhoc Dashboard" sheetId="3" r:id="Rf1fd88f624104ae7"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1629,7 +1629,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R820b2fc9c1234442"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rd2a8519470dd402f"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1659,7 +1659,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R767c206040624673"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R37188d9774c84e6b"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1689,7 +1689,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R2f051d918066412f"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rdac270d4f4fd44af"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1724,7 +1724,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R9251155e07884699"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rc6586b49a59e4dfe"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1759,7 +1759,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R572456a4f56549cf"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rcb5ef71c409e4b7a"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2556,7 +2556,7 @@
     <x:mergeCell ref="A44:F44"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2454ac82a7754661"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R08da6026d5b54c28"/>
 </x:worksheet>
 </file>
 
@@ -3070,7 +3070,7 @@
     <x:mergeCell ref="H27:L27"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R353c40240280451f"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R951c3e55660a4891"/>
 </x:worksheet>
 </file>
 
@@ -3483,6 +3483,6 @@
     <x:mergeCell ref="A20:H20"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8f64f97ee40e493a"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra752c271b1694709"/>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Finalize MVA cloud reports and release artifacts (#2)
Co-authored-by: Mohammed Shahid <DrHayabusa@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/output/excel/mva_crowdstrike_final_team_sample.xlsx
+++ b/output/excel/mva_crowdstrike_final_team_sample.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive Dashboard" sheetId="1" r:id="Racf03b5a09da4987"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monthly Dashboard" sheetId="2" r:id="R5239d2cdeec04484"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Adhoc Dashboard" sheetId="3" r:id="R04e6a03276284a69"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive Dashboard" sheetId="1" r:id="R674dcd0a08cc4d7d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monthly Dashboard" sheetId="2" r:id="Rb7e7139243e44fcf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Adhoc Dashboard" sheetId="3" r:id="Rf1fd88f624104ae7"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1629,7 +1629,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R820b2fc9c1234442"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rd2a8519470dd402f"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1659,7 +1659,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R767c206040624673"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R37188d9774c84e6b"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1689,7 +1689,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R2f051d918066412f"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rdac270d4f4fd44af"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1724,7 +1724,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R9251155e07884699"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rc6586b49a59e4dfe"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1759,7 +1759,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R572456a4f56549cf"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rcb5ef71c409e4b7a"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2556,7 +2556,7 @@
     <x:mergeCell ref="A44:F44"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2454ac82a7754661"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R08da6026d5b54c28"/>
 </x:worksheet>
 </file>
 
@@ -3070,7 +3070,7 @@
     <x:mergeCell ref="H27:L27"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R353c40240280451f"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R951c3e55660a4891"/>
 </x:worksheet>
 </file>
 
@@ -3483,6 +3483,6 @@
     <x:mergeCell ref="A20:H20"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8f64f97ee40e493a"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra752c271b1694709"/>
 </x:worksheet>
 </file>
</xml_diff>